<commit_message>
se añadio nueva info a los jgdores
</commit_message>
<xml_diff>
--- a/Ids Ligas, Equipo.xlsx
+++ b/Ids Ligas, Equipo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MATEO\Videos\JAVASCRIPT\APIs\sports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3986077-E6EC-452D-AD79-4F08E2143EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F09E4AD-8C20-435B-81BE-4C805F00D362}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1776" yWindow="6840" windowWidth="10428" windowHeight="5268" xr2:uid="{13C4450F-79C6-46C9-9EE9-A368FE75A248}"/>
+    <workbookView xWindow="744" yWindow="7476" windowWidth="11172" windowHeight="5364" xr2:uid="{13C4450F-79C6-46C9-9EE9-A368FE75A248}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="283">
   <si>
     <t>id</t>
   </si>
@@ -865,6 +865,15 @@
   </si>
   <si>
     <t>Supercopa de España</t>
+  </si>
+  <si>
+    <t>Eurocopa</t>
+  </si>
+  <si>
+    <t>Liga de Campeones de la AFC</t>
+  </si>
+  <si>
+    <t>Liga Profesional Saudi</t>
   </si>
 </sst>
 </file>
@@ -946,9 +955,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -957,6 +963,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1276,7 +1285,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="18.88671875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" style="4" customWidth="1"/>
     <col min="4" max="4" width="11.5546875" style="1"/>
     <col min="5" max="5" width="17.77734375" style="1" customWidth="1"/>
     <col min="7" max="7" width="11.5546875" style="2"/>
@@ -1284,30 +1293,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="D1" s="3" t="s">
+      <c r="B1" s="6"/>
+      <c r="D1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="3"/>
-      <c r="G1" s="3" t="s">
+      <c r="E1" s="6"/>
+      <c r="G1" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="H1" s="3"/>
+      <c r="H1" s="6"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>2</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -1321,7 +1330,7 @@
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="1">
@@ -1341,7 +1350,7 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="1">
@@ -1361,7 +1370,7 @@
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="1">
@@ -1381,7 +1390,7 @@
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="1">
@@ -1401,7 +1410,7 @@
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="1">
@@ -1421,7 +1430,7 @@
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="1">
@@ -1441,7 +1450,7 @@
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="1">
@@ -1461,7 +1470,7 @@
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="1">
@@ -1481,7 +1490,7 @@
       <c r="A11" s="1">
         <v>9</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="1">
@@ -1501,7 +1510,7 @@
       <c r="A12" s="1">
         <v>10</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="1">
@@ -1521,7 +1530,7 @@
       <c r="A13" s="1">
         <v>11</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D13" s="1">
@@ -1541,7 +1550,7 @@
       <c r="A14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D14" s="1">
@@ -1561,7 +1570,7 @@
       <c r="A15" s="1">
         <v>13</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D15" s="1">
@@ -1581,7 +1590,7 @@
       <c r="A16" s="1">
         <v>14</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="1">
@@ -1601,7 +1610,7 @@
       <c r="A17" s="1">
         <v>15</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D17" s="1">
@@ -1621,7 +1630,7 @@
       <c r="A18" s="1">
         <v>16</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D18" s="1">
@@ -1641,7 +1650,7 @@
       <c r="A19" s="1">
         <v>17</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D19" s="1">
@@ -1661,7 +1670,7 @@
       <c r="A20" s="1">
         <v>18</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D20" s="1">
@@ -1681,7 +1690,7 @@
       <c r="A21" s="1">
         <v>19</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="1">
@@ -1701,7 +1710,7 @@
       <c r="A22" s="1">
         <v>20</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>22</v>
       </c>
       <c r="D22" s="1">
@@ -1721,7 +1730,7 @@
       <c r="A23" s="1">
         <v>21</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D23" s="1">
@@ -1741,10 +1750,10 @@
       <c r="A24" s="1">
         <v>22</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="5">
         <v>2001</v>
       </c>
       <c r="E24" s="1" t="s">
@@ -1759,10 +1768,10 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
-        <v>24</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>279</v>
+        <v>23</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>280</v>
       </c>
       <c r="D25" s="1">
         <v>2002</v>
@@ -1778,6 +1787,12 @@
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>24</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>279</v>
+      </c>
       <c r="D26" s="1">
         <v>2003</v>
       </c>
@@ -1791,7 +1806,13 @@
         <v>90</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>25</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>281</v>
+      </c>
       <c r="D27" s="1">
         <v>2004</v>
       </c>
@@ -1806,6 +1827,12 @@
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>26</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>282</v>
+      </c>
       <c r="D28" s="1">
         <v>2005</v>
       </c>

</xml_diff>

<commit_message>
en jugadores_fu.js se cambio el orden la tabla del historial de jugadores
</commit_message>
<xml_diff>
--- a/Ids Ligas, Equipo.xlsx
+++ b/Ids Ligas, Equipo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MATEO\Videos\JAVASCRIPT\APIs\sports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F09E4AD-8C20-435B-81BE-4C805F00D362}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DAA8C2A-90CC-4413-BDBF-DC7550F8AC62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="744" yWindow="7476" windowWidth="11172" windowHeight="5364" xr2:uid="{13C4450F-79C6-46C9-9EE9-A368FE75A248}"/>
+    <workbookView xWindow="744" yWindow="6876" windowWidth="11172" windowHeight="5364" xr2:uid="{13C4450F-79C6-46C9-9EE9-A368FE75A248}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="284">
   <si>
     <t>id</t>
   </si>
@@ -874,6 +874,9 @@
   </si>
   <si>
     <t>Liga Profesional Saudi</t>
+  </si>
+  <si>
+    <t>Copa Africana de Naciones</t>
   </si>
 </sst>
 </file>
@@ -1846,7 +1849,13 @@
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>27</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>283</v>
+      </c>
       <c r="D29" s="1">
         <v>2006</v>
       </c>

</xml_diff>

<commit_message>
se mejoro la funcion historialTabla
</commit_message>
<xml_diff>
--- a/Ids Ligas, Equipo.xlsx
+++ b/Ids Ligas, Equipo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MATEO\Videos\JAVASCRIPT\APIs\sports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DAA8C2A-90CC-4413-BDBF-DC7550F8AC62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3A65FE3-CAEA-405A-95B6-04E4C2C70239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="744" yWindow="6876" windowWidth="11172" windowHeight="5364" xr2:uid="{13C4450F-79C6-46C9-9EE9-A368FE75A248}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{13C4450F-79C6-46C9-9EE9-A368FE75A248}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="410">
   <si>
     <t>id</t>
   </si>
@@ -877,6 +877,384 @@
   </si>
   <si>
     <t>Copa Africana de Naciones</t>
+  </si>
+  <si>
+    <t>Eurocopa sub-21</t>
+  </si>
+  <si>
+    <t>Bayern Munich</t>
+  </si>
+  <si>
+    <t>Borussia Dortmund</t>
+  </si>
+  <si>
+    <t>RB Leipzig</t>
+  </si>
+  <si>
+    <t>Bayer Leverkusen</t>
+  </si>
+  <si>
+    <t>Borussia Monchengladbach</t>
+  </si>
+  <si>
+    <t>Schalke 04</t>
+  </si>
+  <si>
+    <t>Eintracht Frankfurt</t>
+  </si>
+  <si>
+    <t>VFL Wolfsburg</t>
+  </si>
+  <si>
+    <t>TSG Hoffenheim</t>
+  </si>
+  <si>
+    <t>SC Freiburg</t>
+  </si>
+  <si>
+    <t>Union Berlin</t>
+  </si>
+  <si>
+    <t>VFB Stuttgart</t>
+  </si>
+  <si>
+    <t>FC Augsburg</t>
+  </si>
+  <si>
+    <t>FSV Mainz 05</t>
+  </si>
+  <si>
+    <t>FC Koln</t>
+  </si>
+  <si>
+    <t>Werder Bremen</t>
+  </si>
+  <si>
+    <t>Hertha Berlin</t>
+  </si>
+  <si>
+    <t>VFL Bochum</t>
+  </si>
+  <si>
+    <t>PSG</t>
+  </si>
+  <si>
+    <t>Olympique de Lyon</t>
+  </si>
+  <si>
+    <t>Olympique de Marsella</t>
+  </si>
+  <si>
+    <t>AS Monaco</t>
+  </si>
+  <si>
+    <t>Lille</t>
+  </si>
+  <si>
+    <t>Stade Rennais</t>
+  </si>
+  <si>
+    <t>Racing Club de Lens</t>
+  </si>
+  <si>
+    <t>Niza</t>
+  </si>
+  <si>
+    <t>Toulouse</t>
+  </si>
+  <si>
+    <t>Le Havre</t>
+  </si>
+  <si>
+    <t>Paris FC</t>
+  </si>
+  <si>
+    <t>Lens FC</t>
+  </si>
+  <si>
+    <t>Angers</t>
+  </si>
+  <si>
+    <t>Metz FC</t>
+  </si>
+  <si>
+    <t>Stade Brestois</t>
+  </si>
+  <si>
+    <t>Nantes FC</t>
+  </si>
+  <si>
+    <t>Lorient FC</t>
+  </si>
+  <si>
+    <t>Auxerre</t>
+  </si>
+  <si>
+    <t>Atalanta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bolonia </t>
+  </si>
+  <si>
+    <t>Cagliari</t>
+  </si>
+  <si>
+    <t>Como</t>
+  </si>
+  <si>
+    <t>Cremonese</t>
+  </si>
+  <si>
+    <t>Fiorentina</t>
+  </si>
+  <si>
+    <t>Genoa</t>
+  </si>
+  <si>
+    <t>Hellas Verona</t>
+  </si>
+  <si>
+    <t>Inter</t>
+  </si>
+  <si>
+    <t>Juventus</t>
+  </si>
+  <si>
+    <t>Lazio</t>
+  </si>
+  <si>
+    <t>Lecce</t>
+  </si>
+  <si>
+    <t>Milan</t>
+  </si>
+  <si>
+    <t>Napoli</t>
+  </si>
+  <si>
+    <t>Parma</t>
+  </si>
+  <si>
+    <t>Pisa</t>
+  </si>
+  <si>
+    <t>Roma</t>
+  </si>
+  <si>
+    <t>Sassuolo</t>
+  </si>
+  <si>
+    <t>Torino</t>
+  </si>
+  <si>
+    <t>Udinese</t>
+  </si>
+  <si>
+    <t>Ajax</t>
+  </si>
+  <si>
+    <t>AZ</t>
+  </si>
+  <si>
+    <t>Excelsior</t>
+  </si>
+  <si>
+    <t>Feyenoord</t>
+  </si>
+  <si>
+    <t>Fortuna Sittard</t>
+  </si>
+  <si>
+    <t>Go Ahead Eagles</t>
+  </si>
+  <si>
+    <t>Groningeen</t>
+  </si>
+  <si>
+    <t>Heerenveen</t>
+  </si>
+  <si>
+    <t>Heracles</t>
+  </si>
+  <si>
+    <t>NAC</t>
+  </si>
+  <si>
+    <t>NEC</t>
+  </si>
+  <si>
+    <t>PSV</t>
+  </si>
+  <si>
+    <t>Sparta Rotterdam</t>
+  </si>
+  <si>
+    <t>SC Telstr</t>
+  </si>
+  <si>
+    <t>Twente</t>
+  </si>
+  <si>
+    <t>Utrecth</t>
+  </si>
+  <si>
+    <t>Volendam</t>
+  </si>
+  <si>
+    <t>Zwolle</t>
+  </si>
+  <si>
+    <t>Arouca</t>
+  </si>
+  <si>
+    <t>AVS</t>
+  </si>
+  <si>
+    <t>Benfica</t>
+  </si>
+  <si>
+    <t>Braga</t>
+  </si>
+  <si>
+    <t>Casa Pia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estoril </t>
+  </si>
+  <si>
+    <t>Estrela Amadora</t>
+  </si>
+  <si>
+    <t>Famalicao</t>
+  </si>
+  <si>
+    <t>Gil Vicente</t>
+  </si>
+  <si>
+    <t>Guimaraes</t>
+  </si>
+  <si>
+    <t>Moreirense</t>
+  </si>
+  <si>
+    <t>Nacional</t>
+  </si>
+  <si>
+    <t>Porto</t>
+  </si>
+  <si>
+    <t>Rio Ave</t>
+  </si>
+  <si>
+    <t>Santa Clara</t>
+  </si>
+  <si>
+    <t>Sporting Lisboa</t>
+  </si>
+  <si>
+    <t>Tondela</t>
+  </si>
+  <si>
+    <t>Anderlecht</t>
+  </si>
+  <si>
+    <t>Antwerp</t>
+  </si>
+  <si>
+    <t>Cercle Brugge</t>
+  </si>
+  <si>
+    <t>Charleroi</t>
+  </si>
+  <si>
+    <t>Club Brujas</t>
+  </si>
+  <si>
+    <t>FC Dender Eh</t>
+  </si>
+  <si>
+    <t>Gent</t>
+  </si>
+  <si>
+    <t>KRC Genk</t>
+  </si>
+  <si>
+    <t>Leuven</t>
+  </si>
+  <si>
+    <t>Mechelen</t>
+  </si>
+  <si>
+    <t>RAAL La Louviare</t>
+  </si>
+  <si>
+    <t>Standard Lieja</t>
+  </si>
+  <si>
+    <t>STVV</t>
+  </si>
+  <si>
+    <t>Union Staint-gilloise</t>
+  </si>
+  <si>
+    <t>Westerlo</t>
+  </si>
+  <si>
+    <t>Zulte Waregem</t>
+  </si>
+  <si>
+    <t>Al Nasrr</t>
+  </si>
+  <si>
+    <t>Al Taawon</t>
+  </si>
+  <si>
+    <t>Al Hilal</t>
+  </si>
+  <si>
+    <t>Al Qadsiah</t>
+  </si>
+  <si>
+    <t>Al ahli Saudi</t>
+  </si>
+  <si>
+    <t>Al khaleej</t>
+  </si>
+  <si>
+    <t>Neom Sports</t>
+  </si>
+  <si>
+    <t>Al ittihad</t>
+  </si>
+  <si>
+    <t>Al Fayha</t>
+  </si>
+  <si>
+    <t>Al Khoolod</t>
+  </si>
+  <si>
+    <t>Al Ettifaq</t>
+  </si>
+  <si>
+    <t>Al Riyadh</t>
+  </si>
+  <si>
+    <t>Al Shabab</t>
+  </si>
+  <si>
+    <t>Al Hazm</t>
+  </si>
+  <si>
+    <t>Al Fateh</t>
+  </si>
+  <si>
+    <t>Al Okhdood</t>
+  </si>
+  <si>
+    <t>Damac</t>
+  </si>
+  <si>
+    <t>Al Najma</t>
   </si>
 </sst>
 </file>
@@ -1290,7 +1668,7 @@
     <col min="1" max="1" width="11.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="18.88671875" style="4" customWidth="1"/>
     <col min="4" max="4" width="11.5546875" style="1"/>
-    <col min="5" max="5" width="17.77734375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="25.77734375" style="1" customWidth="1"/>
     <col min="7" max="7" width="11.5546875" style="2"/>
     <col min="8" max="8" width="23.5546875" style="2" customWidth="1"/>
   </cols>
@@ -1870,6 +2248,12 @@
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
+        <v>28</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>284</v>
+      </c>
       <c r="D30" s="1">
         <v>2007</v>
       </c>
@@ -2066,6 +2450,12 @@
       </c>
     </row>
     <row r="44" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D44" s="1">
+        <v>3001</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="G44" s="1">
         <v>42</v>
       </c>
@@ -2074,6 +2464,12 @@
       </c>
     </row>
     <row r="45" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D45" s="1">
+        <v>3002</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>286</v>
+      </c>
       <c r="G45" s="1">
         <v>43</v>
       </c>
@@ -2082,6 +2478,12 @@
       </c>
     </row>
     <row r="46" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D46" s="1">
+        <v>3003</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>287</v>
+      </c>
       <c r="G46" s="1">
         <v>44</v>
       </c>
@@ -2090,6 +2492,12 @@
       </c>
     </row>
     <row r="47" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D47" s="1">
+        <v>3004</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>288</v>
+      </c>
       <c r="G47" s="1">
         <v>45</v>
       </c>
@@ -2098,6 +2506,12 @@
       </c>
     </row>
     <row r="48" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D48" s="1">
+        <v>3005</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>289</v>
+      </c>
       <c r="G48" s="1">
         <v>46</v>
       </c>
@@ -2105,7 +2519,13 @@
         <v>112</v>
       </c>
     </row>
-    <row r="49" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D49" s="1">
+        <v>3006</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>290</v>
+      </c>
       <c r="G49" s="1">
         <v>47</v>
       </c>
@@ -2113,7 +2533,13 @@
         <v>113</v>
       </c>
     </row>
-    <row r="50" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D50" s="1">
+        <v>3007</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>291</v>
+      </c>
       <c r="G50" s="1">
         <v>48</v>
       </c>
@@ -2121,7 +2547,13 @@
         <v>114</v>
       </c>
     </row>
-    <row r="51" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D51" s="1">
+        <v>3008</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>292</v>
+      </c>
       <c r="G51" s="1">
         <v>49</v>
       </c>
@@ -2129,7 +2561,13 @@
         <v>115</v>
       </c>
     </row>
-    <row r="52" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D52" s="1">
+        <v>3009</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>293</v>
+      </c>
       <c r="G52" s="1">
         <v>50</v>
       </c>
@@ -2137,7 +2575,13 @@
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D53" s="1">
+        <v>3010</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>294</v>
+      </c>
       <c r="G53" s="1">
         <v>51</v>
       </c>
@@ -2145,7 +2589,13 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D54" s="1">
+        <v>3011</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>295</v>
+      </c>
       <c r="G54" s="1">
         <v>52</v>
       </c>
@@ -2153,7 +2603,13 @@
         <v>118</v>
       </c>
     </row>
-    <row r="55" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D55" s="1">
+        <v>3012</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>296</v>
+      </c>
       <c r="G55" s="1">
         <v>53</v>
       </c>
@@ -2161,7 +2617,13 @@
         <v>119</v>
       </c>
     </row>
-    <row r="56" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D56" s="1">
+        <v>3013</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>297</v>
+      </c>
       <c r="G56" s="1">
         <v>54</v>
       </c>
@@ -2169,7 +2631,13 @@
         <v>120</v>
       </c>
     </row>
-    <row r="57" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D57" s="1">
+        <v>3014</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>298</v>
+      </c>
       <c r="G57" s="1">
         <v>55</v>
       </c>
@@ -2177,7 +2645,13 @@
         <v>121</v>
       </c>
     </row>
-    <row r="58" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D58" s="1">
+        <v>3015</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>299</v>
+      </c>
       <c r="G58" s="1">
         <v>56</v>
       </c>
@@ -2185,7 +2659,13 @@
         <v>122</v>
       </c>
     </row>
-    <row r="59" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D59" s="1">
+        <v>3016</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>300</v>
+      </c>
       <c r="G59" s="1">
         <v>57</v>
       </c>
@@ -2193,7 +2673,13 @@
         <v>123</v>
       </c>
     </row>
-    <row r="60" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D60" s="1">
+        <v>3017</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>301</v>
+      </c>
       <c r="G60" s="1">
         <v>58</v>
       </c>
@@ -2201,7 +2687,13 @@
         <v>124</v>
       </c>
     </row>
-    <row r="61" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D61" s="1">
+        <v>3018</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>302</v>
+      </c>
       <c r="G61" s="1">
         <v>59</v>
       </c>
@@ -2209,7 +2701,13 @@
         <v>125</v>
       </c>
     </row>
-    <row r="62" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D62" s="1">
+        <v>4001</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>303</v>
+      </c>
       <c r="G62" s="1">
         <v>60</v>
       </c>
@@ -2217,7 +2715,13 @@
         <v>126</v>
       </c>
     </row>
-    <row r="63" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D63" s="1">
+        <v>4002</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>305</v>
+      </c>
       <c r="G63" s="1">
         <v>61</v>
       </c>
@@ -2225,7 +2729,13 @@
         <v>127</v>
       </c>
     </row>
-    <row r="64" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D64" s="1">
+        <v>4003</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>304</v>
+      </c>
       <c r="G64" s="1">
         <v>62</v>
       </c>
@@ -2233,7 +2743,13 @@
         <v>128</v>
       </c>
     </row>
-    <row r="65" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D65" s="1">
+        <v>4004</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>306</v>
+      </c>
       <c r="G65" s="1">
         <v>63</v>
       </c>
@@ -2241,7 +2757,13 @@
         <v>129</v>
       </c>
     </row>
-    <row r="66" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D66" s="1">
+        <v>4005</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>307</v>
+      </c>
       <c r="G66" s="1">
         <v>64</v>
       </c>
@@ -2249,7 +2771,13 @@
         <v>130</v>
       </c>
     </row>
-    <row r="67" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D67" s="1">
+        <v>4006</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>308</v>
+      </c>
       <c r="G67" s="1">
         <v>65</v>
       </c>
@@ -2257,7 +2785,13 @@
         <v>131</v>
       </c>
     </row>
-    <row r="68" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D68" s="1">
+        <v>4007</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>309</v>
+      </c>
       <c r="G68" s="1">
         <v>66</v>
       </c>
@@ -2265,7 +2799,13 @@
         <v>132</v>
       </c>
     </row>
-    <row r="69" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D69" s="1">
+        <v>4008</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>310</v>
+      </c>
       <c r="G69" s="1">
         <v>67</v>
       </c>
@@ -2273,7 +2813,13 @@
         <v>133</v>
       </c>
     </row>
-    <row r="70" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D70" s="1">
+        <v>4009</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>311</v>
+      </c>
       <c r="G70" s="1">
         <v>68</v>
       </c>
@@ -2281,7 +2827,13 @@
         <v>134</v>
       </c>
     </row>
-    <row r="71" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D71" s="1">
+        <v>4010</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>312</v>
+      </c>
       <c r="G71" s="1">
         <v>69</v>
       </c>
@@ -2289,7 +2841,13 @@
         <v>135</v>
       </c>
     </row>
-    <row r="72" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D72" s="1">
+        <v>4011</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>313</v>
+      </c>
       <c r="G72" s="1">
         <v>70</v>
       </c>
@@ -2297,7 +2855,13 @@
         <v>136</v>
       </c>
     </row>
-    <row r="73" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D73" s="1">
+        <v>4012</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>314</v>
+      </c>
       <c r="G73" s="1">
         <v>71</v>
       </c>
@@ -2305,7 +2869,13 @@
         <v>137</v>
       </c>
     </row>
-    <row r="74" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D74" s="1">
+        <v>4013</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>315</v>
+      </c>
       <c r="G74" s="1">
         <v>72</v>
       </c>
@@ -2313,7 +2883,13 @@
         <v>138</v>
       </c>
     </row>
-    <row r="75" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D75" s="1">
+        <v>4014</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>316</v>
+      </c>
       <c r="G75" s="1">
         <v>73</v>
       </c>
@@ -2321,7 +2897,13 @@
         <v>139</v>
       </c>
     </row>
-    <row r="76" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D76" s="1">
+        <v>4015</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>317</v>
+      </c>
       <c r="G76" s="1">
         <v>74</v>
       </c>
@@ -2329,7 +2911,13 @@
         <v>140</v>
       </c>
     </row>
-    <row r="77" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D77" s="1">
+        <v>4016</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>318</v>
+      </c>
       <c r="G77" s="1">
         <v>75</v>
       </c>
@@ -2337,7 +2925,13 @@
         <v>141</v>
       </c>
     </row>
-    <row r="78" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D78" s="1">
+        <v>4017</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>319</v>
+      </c>
       <c r="G78" s="1">
         <v>76</v>
       </c>
@@ -2345,7 +2939,13 @@
         <v>142</v>
       </c>
     </row>
-    <row r="79" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D79" s="1">
+        <v>4018</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>320</v>
+      </c>
       <c r="G79" s="1">
         <v>77</v>
       </c>
@@ -2353,7 +2953,13 @@
         <v>143</v>
       </c>
     </row>
-    <row r="80" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D80" s="1">
+        <v>5001</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>321</v>
+      </c>
       <c r="G80" s="1">
         <v>78</v>
       </c>
@@ -2361,7 +2967,13 @@
         <v>144</v>
       </c>
     </row>
-    <row r="81" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D81" s="1">
+        <v>5002</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>322</v>
+      </c>
       <c r="G81" s="1">
         <v>79</v>
       </c>
@@ -2369,7 +2981,13 @@
         <v>145</v>
       </c>
     </row>
-    <row r="82" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D82" s="1">
+        <v>5003</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>323</v>
+      </c>
       <c r="G82" s="1">
         <v>80</v>
       </c>
@@ -2377,7 +2995,13 @@
         <v>146</v>
       </c>
     </row>
-    <row r="83" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D83" s="1">
+        <v>5004</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>324</v>
+      </c>
       <c r="G83" s="1">
         <v>81</v>
       </c>
@@ -2385,7 +3009,13 @@
         <v>147</v>
       </c>
     </row>
-    <row r="84" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D84" s="1">
+        <v>5005</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>325</v>
+      </c>
       <c r="G84" s="1">
         <v>82</v>
       </c>
@@ -2393,7 +3023,13 @@
         <v>148</v>
       </c>
     </row>
-    <row r="85" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D85" s="1">
+        <v>5006</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>326</v>
+      </c>
       <c r="G85" s="1">
         <v>83</v>
       </c>
@@ -2401,7 +3037,13 @@
         <v>149</v>
       </c>
     </row>
-    <row r="86" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="86" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D86" s="1">
+        <v>5007</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>327</v>
+      </c>
       <c r="G86" s="1">
         <v>84</v>
       </c>
@@ -2409,7 +3051,13 @@
         <v>150</v>
       </c>
     </row>
-    <row r="87" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="87" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D87" s="1">
+        <v>5008</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>328</v>
+      </c>
       <c r="G87" s="1">
         <v>85</v>
       </c>
@@ -2417,7 +3065,13 @@
         <v>151</v>
       </c>
     </row>
-    <row r="88" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D88" s="1">
+        <v>5009</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>329</v>
+      </c>
       <c r="G88" s="1">
         <v>86</v>
       </c>
@@ -2425,7 +3079,13 @@
         <v>152</v>
       </c>
     </row>
-    <row r="89" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="89" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D89" s="1">
+        <v>5010</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>330</v>
+      </c>
       <c r="G89" s="1">
         <v>87</v>
       </c>
@@ -2433,7 +3093,13 @@
         <v>153</v>
       </c>
     </row>
-    <row r="90" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D90" s="1">
+        <v>5011</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>331</v>
+      </c>
       <c r="G90" s="1">
         <v>88</v>
       </c>
@@ -2441,7 +3107,13 @@
         <v>154</v>
       </c>
     </row>
-    <row r="91" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="91" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D91" s="1">
+        <v>5012</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>332</v>
+      </c>
       <c r="G91" s="1">
         <v>89</v>
       </c>
@@ -2449,7 +3121,13 @@
         <v>155</v>
       </c>
     </row>
-    <row r="92" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D92" s="1">
+        <v>5013</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>333</v>
+      </c>
       <c r="G92" s="1">
         <v>90</v>
       </c>
@@ -2457,7 +3135,13 @@
         <v>156</v>
       </c>
     </row>
-    <row r="93" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D93" s="1">
+        <v>5014</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>334</v>
+      </c>
       <c r="G93" s="1">
         <v>91</v>
       </c>
@@ -2465,7 +3149,13 @@
         <v>157</v>
       </c>
     </row>
-    <row r="94" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D94" s="1">
+        <v>5015</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>335</v>
+      </c>
       <c r="G94" s="1">
         <v>92</v>
       </c>
@@ -2473,7 +3163,13 @@
         <v>158</v>
       </c>
     </row>
-    <row r="95" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D95" s="1">
+        <v>5016</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>336</v>
+      </c>
       <c r="G95" s="1">
         <v>93</v>
       </c>
@@ -2481,7 +3177,13 @@
         <v>159</v>
       </c>
     </row>
-    <row r="96" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D96" s="1">
+        <v>5017</v>
+      </c>
+      <c r="E96" s="1" t="s">
+        <v>337</v>
+      </c>
       <c r="G96" s="1">
         <v>94</v>
       </c>
@@ -2489,7 +3191,13 @@
         <v>160</v>
       </c>
     </row>
-    <row r="97" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D97" s="1">
+        <v>5018</v>
+      </c>
+      <c r="E97" s="1" t="s">
+        <v>338</v>
+      </c>
       <c r="G97" s="1">
         <v>95</v>
       </c>
@@ -2497,7 +3205,13 @@
         <v>161</v>
       </c>
     </row>
-    <row r="98" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D98" s="1">
+        <v>5019</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>339</v>
+      </c>
       <c r="G98" s="1">
         <v>96</v>
       </c>
@@ -2505,7 +3219,13 @@
         <v>162</v>
       </c>
     </row>
-    <row r="99" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D99" s="1">
+        <v>5020</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>340</v>
+      </c>
       <c r="G99" s="1">
         <v>97</v>
       </c>
@@ -2513,7 +3233,13 @@
         <v>163</v>
       </c>
     </row>
-    <row r="100" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D100" s="1">
+        <v>6001</v>
+      </c>
+      <c r="E100" s="1" t="s">
+        <v>341</v>
+      </c>
       <c r="G100" s="1">
         <v>98</v>
       </c>
@@ -2521,7 +3247,13 @@
         <v>164</v>
       </c>
     </row>
-    <row r="101" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D101" s="1">
+        <v>6002</v>
+      </c>
+      <c r="E101" s="1" t="s">
+        <v>342</v>
+      </c>
       <c r="G101" s="1">
         <v>99</v>
       </c>
@@ -2529,7 +3261,13 @@
         <v>165</v>
       </c>
     </row>
-    <row r="102" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D102" s="1">
+        <v>6003</v>
+      </c>
+      <c r="E102" s="1" t="s">
+        <v>343</v>
+      </c>
       <c r="G102" s="1">
         <v>100</v>
       </c>
@@ -2537,7 +3275,13 @@
         <v>166</v>
       </c>
     </row>
-    <row r="103" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D103" s="1">
+        <v>6004</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>344</v>
+      </c>
       <c r="G103" s="1">
         <v>101</v>
       </c>
@@ -2545,7 +3289,13 @@
         <v>167</v>
       </c>
     </row>
-    <row r="104" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D104" s="1">
+        <v>6005</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>345</v>
+      </c>
       <c r="G104" s="1">
         <v>102</v>
       </c>
@@ -2553,7 +3303,13 @@
         <v>168</v>
       </c>
     </row>
-    <row r="105" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D105" s="1">
+        <v>6006</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>346</v>
+      </c>
       <c r="G105" s="1">
         <v>103</v>
       </c>
@@ -2561,7 +3317,13 @@
         <v>169</v>
       </c>
     </row>
-    <row r="106" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D106" s="1">
+        <v>6007</v>
+      </c>
+      <c r="E106" s="1" t="s">
+        <v>347</v>
+      </c>
       <c r="G106" s="1">
         <v>104</v>
       </c>
@@ -2569,7 +3331,13 @@
         <v>170</v>
       </c>
     </row>
-    <row r="107" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D107" s="1">
+        <v>6008</v>
+      </c>
+      <c r="E107" s="1" t="s">
+        <v>348</v>
+      </c>
       <c r="G107" s="1">
         <v>105</v>
       </c>
@@ -2577,7 +3345,13 @@
         <v>171</v>
       </c>
     </row>
-    <row r="108" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D108" s="1">
+        <v>6009</v>
+      </c>
+      <c r="E108" s="1" t="s">
+        <v>349</v>
+      </c>
       <c r="G108" s="1">
         <v>106</v>
       </c>
@@ -2585,7 +3359,13 @@
         <v>172</v>
       </c>
     </row>
-    <row r="109" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D109" s="1">
+        <v>6010</v>
+      </c>
+      <c r="E109" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="G109" s="1">
         <v>107</v>
       </c>
@@ -2593,7 +3373,13 @@
         <v>173</v>
       </c>
     </row>
-    <row r="110" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D110" s="1">
+        <v>6011</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="G110" s="1">
         <v>108</v>
       </c>
@@ -2601,7 +3387,13 @@
         <v>174</v>
       </c>
     </row>
-    <row r="111" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="111" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D111" s="1">
+        <v>6012</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>352</v>
+      </c>
       <c r="G111" s="1">
         <v>109</v>
       </c>
@@ -2609,7 +3401,13 @@
         <v>175</v>
       </c>
     </row>
-    <row r="112" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D112" s="1">
+        <v>6013</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>353</v>
+      </c>
       <c r="G112" s="1">
         <v>110</v>
       </c>
@@ -2617,7 +3415,13 @@
         <v>176</v>
       </c>
     </row>
-    <row r="113" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="113" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D113" s="1">
+        <v>6014</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>354</v>
+      </c>
       <c r="G113" s="1">
         <v>111</v>
       </c>
@@ -2625,7 +3429,13 @@
         <v>177</v>
       </c>
     </row>
-    <row r="114" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="114" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D114" s="1">
+        <v>6015</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>355</v>
+      </c>
       <c r="G114" s="1">
         <v>112</v>
       </c>
@@ -2633,7 +3443,13 @@
         <v>178</v>
       </c>
     </row>
-    <row r="115" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="115" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D115" s="1">
+        <v>6016</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>356</v>
+      </c>
       <c r="G115" s="1">
         <v>113</v>
       </c>
@@ -2641,7 +3457,13 @@
         <v>179</v>
       </c>
     </row>
-    <row r="116" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="116" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D116" s="1">
+        <v>6017</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>357</v>
+      </c>
       <c r="G116" s="1">
         <v>114</v>
       </c>
@@ -2649,7 +3471,13 @@
         <v>180</v>
       </c>
     </row>
-    <row r="117" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="117" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D117" s="1">
+        <v>6018</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>358</v>
+      </c>
       <c r="G117" s="1">
         <v>115</v>
       </c>
@@ -2657,7 +3485,13 @@
         <v>181</v>
       </c>
     </row>
-    <row r="118" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="118" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D118" s="1">
+        <v>7001</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>359</v>
+      </c>
       <c r="G118" s="1">
         <v>116</v>
       </c>
@@ -2665,7 +3499,13 @@
         <v>182</v>
       </c>
     </row>
-    <row r="119" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="119" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D119" s="1">
+        <v>7002</v>
+      </c>
+      <c r="E119" s="1" t="s">
+        <v>360</v>
+      </c>
       <c r="G119" s="1">
         <v>117</v>
       </c>
@@ -2673,7 +3513,13 @@
         <v>183</v>
       </c>
     </row>
-    <row r="120" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="120" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D120" s="1">
+        <v>7003</v>
+      </c>
+      <c r="E120" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="G120" s="1">
         <v>118</v>
       </c>
@@ -2681,7 +3527,13 @@
         <v>184</v>
       </c>
     </row>
-    <row r="121" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="121" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D121" s="1">
+        <v>7004</v>
+      </c>
+      <c r="E121" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="G121" s="1">
         <v>119</v>
       </c>
@@ -2689,7 +3541,13 @@
         <v>185</v>
       </c>
     </row>
-    <row r="122" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="122" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D122" s="1">
+        <v>7005</v>
+      </c>
+      <c r="E122" s="1" t="s">
+        <v>363</v>
+      </c>
       <c r="G122" s="1">
         <v>120</v>
       </c>
@@ -2697,7 +3555,13 @@
         <v>186</v>
       </c>
     </row>
-    <row r="123" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="123" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D123" s="1">
+        <v>7006</v>
+      </c>
+      <c r="E123" s="1" t="s">
+        <v>364</v>
+      </c>
       <c r="G123" s="1">
         <v>121</v>
       </c>
@@ -2705,7 +3569,13 @@
         <v>187</v>
       </c>
     </row>
-    <row r="124" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="124" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D124" s="1">
+        <v>7007</v>
+      </c>
+      <c r="E124" s="1" t="s">
+        <v>365</v>
+      </c>
       <c r="G124" s="1">
         <v>122</v>
       </c>
@@ -2713,7 +3583,13 @@
         <v>188</v>
       </c>
     </row>
-    <row r="125" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="125" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D125" s="1">
+        <v>7008</v>
+      </c>
+      <c r="E125" s="1" t="s">
+        <v>366</v>
+      </c>
       <c r="G125" s="1">
         <v>123</v>
       </c>
@@ -2721,7 +3597,13 @@
         <v>189</v>
       </c>
     </row>
-    <row r="126" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="126" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D126" s="1">
+        <v>7009</v>
+      </c>
+      <c r="E126" s="1" t="s">
+        <v>367</v>
+      </c>
       <c r="G126" s="1">
         <v>124</v>
       </c>
@@ -2729,7 +3611,13 @@
         <v>190</v>
       </c>
     </row>
-    <row r="127" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="127" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D127" s="1">
+        <v>7010</v>
+      </c>
+      <c r="E127" s="1" t="s">
+        <v>368</v>
+      </c>
       <c r="G127" s="1">
         <v>125</v>
       </c>
@@ -2737,7 +3625,13 @@
         <v>191</v>
       </c>
     </row>
-    <row r="128" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="128" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D128" s="1">
+        <v>7011</v>
+      </c>
+      <c r="E128" s="1" t="s">
+        <v>369</v>
+      </c>
       <c r="G128" s="1">
         <v>126</v>
       </c>
@@ -2745,7 +3639,13 @@
         <v>192</v>
       </c>
     </row>
-    <row r="129" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="129" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D129" s="1">
+        <v>7012</v>
+      </c>
+      <c r="E129" s="1" t="s">
+        <v>370</v>
+      </c>
       <c r="G129" s="1">
         <v>127</v>
       </c>
@@ -2753,7 +3653,13 @@
         <v>193</v>
       </c>
     </row>
-    <row r="130" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="130" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D130" s="1">
+        <v>7013</v>
+      </c>
+      <c r="E130" s="1" t="s">
+        <v>371</v>
+      </c>
       <c r="G130" s="1">
         <v>128</v>
       </c>
@@ -2761,7 +3667,13 @@
         <v>194</v>
       </c>
     </row>
-    <row r="131" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="131" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D131" s="1">
+        <v>7014</v>
+      </c>
+      <c r="E131" s="1" t="s">
+        <v>372</v>
+      </c>
       <c r="G131" s="1">
         <v>129</v>
       </c>
@@ -2769,7 +3681,13 @@
         <v>195</v>
       </c>
     </row>
-    <row r="132" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="132" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D132" s="1">
+        <v>7015</v>
+      </c>
+      <c r="E132" s="1" t="s">
+        <v>373</v>
+      </c>
       <c r="G132" s="1">
         <v>130</v>
       </c>
@@ -2777,7 +3695,13 @@
         <v>196</v>
       </c>
     </row>
-    <row r="133" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="133" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D133" s="1">
+        <v>7016</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>374</v>
+      </c>
       <c r="G133" s="1">
         <v>131</v>
       </c>
@@ -2785,7 +3709,13 @@
         <v>197</v>
       </c>
     </row>
-    <row r="134" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="134" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D134" s="1">
+        <v>7017</v>
+      </c>
+      <c r="E134" s="1" t="s">
+        <v>375</v>
+      </c>
       <c r="G134" s="1">
         <v>132</v>
       </c>
@@ -2793,7 +3723,13 @@
         <v>198</v>
       </c>
     </row>
-    <row r="135" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="135" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D135" s="1">
+        <v>8001</v>
+      </c>
+      <c r="E135" s="1" t="s">
+        <v>376</v>
+      </c>
       <c r="G135" s="1">
         <v>133</v>
       </c>
@@ -2801,7 +3737,13 @@
         <v>199</v>
       </c>
     </row>
-    <row r="136" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="136" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D136" s="1">
+        <v>8002</v>
+      </c>
+      <c r="E136" s="1" t="s">
+        <v>377</v>
+      </c>
       <c r="G136" s="1">
         <v>134</v>
       </c>
@@ -2809,7 +3751,13 @@
         <v>200</v>
       </c>
     </row>
-    <row r="137" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="137" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D137" s="1">
+        <v>8003</v>
+      </c>
+      <c r="E137" s="1" t="s">
+        <v>378</v>
+      </c>
       <c r="G137" s="1">
         <v>135</v>
       </c>
@@ -2817,7 +3765,13 @@
         <v>201</v>
       </c>
     </row>
-    <row r="138" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="138" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D138" s="1">
+        <v>8004</v>
+      </c>
+      <c r="E138" s="1" t="s">
+        <v>379</v>
+      </c>
       <c r="G138" s="1">
         <v>136</v>
       </c>
@@ -2825,7 +3779,13 @@
         <v>202</v>
       </c>
     </row>
-    <row r="139" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="139" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D139" s="1">
+        <v>8005</v>
+      </c>
+      <c r="E139" s="1" t="s">
+        <v>380</v>
+      </c>
       <c r="G139" s="1">
         <v>137</v>
       </c>
@@ -2833,7 +3793,13 @@
         <v>203</v>
       </c>
     </row>
-    <row r="140" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="140" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D140" s="1">
+        <v>8006</v>
+      </c>
+      <c r="E140" s="1" t="s">
+        <v>381</v>
+      </c>
       <c r="G140" s="1">
         <v>138</v>
       </c>
@@ -2841,7 +3807,13 @@
         <v>204</v>
       </c>
     </row>
-    <row r="141" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="141" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D141" s="1">
+        <v>8007</v>
+      </c>
+      <c r="E141" s="1" t="s">
+        <v>382</v>
+      </c>
       <c r="G141" s="1">
         <v>139</v>
       </c>
@@ -2849,7 +3821,13 @@
         <v>205</v>
       </c>
     </row>
-    <row r="142" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="142" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D142" s="1">
+        <v>8008</v>
+      </c>
+      <c r="E142" s="1" t="s">
+        <v>383</v>
+      </c>
       <c r="G142" s="1">
         <v>140</v>
       </c>
@@ -2857,7 +3835,13 @@
         <v>206</v>
       </c>
     </row>
-    <row r="143" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="143" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D143" s="1">
+        <v>8009</v>
+      </c>
+      <c r="E143" s="1" t="s">
+        <v>384</v>
+      </c>
       <c r="G143" s="1">
         <v>141</v>
       </c>
@@ -2865,7 +3849,13 @@
         <v>207</v>
       </c>
     </row>
-    <row r="144" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="144" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D144" s="1">
+        <v>8010</v>
+      </c>
+      <c r="E144" s="1" t="s">
+        <v>385</v>
+      </c>
       <c r="G144" s="1">
         <v>142</v>
       </c>
@@ -2873,7 +3863,13 @@
         <v>208</v>
       </c>
     </row>
-    <row r="145" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="145" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D145" s="1">
+        <v>8011</v>
+      </c>
+      <c r="E145" s="1" t="s">
+        <v>386</v>
+      </c>
       <c r="G145" s="1">
         <v>143</v>
       </c>
@@ -2881,7 +3877,13 @@
         <v>209</v>
       </c>
     </row>
-    <row r="146" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="146" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D146" s="1">
+        <v>8012</v>
+      </c>
+      <c r="E146" s="1" t="s">
+        <v>387</v>
+      </c>
       <c r="G146" s="1">
         <v>144</v>
       </c>
@@ -2889,7 +3891,13 @@
         <v>210</v>
       </c>
     </row>
-    <row r="147" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="147" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D147" s="1">
+        <v>8013</v>
+      </c>
+      <c r="E147" s="1" t="s">
+        <v>388</v>
+      </c>
       <c r="G147" s="1">
         <v>145</v>
       </c>
@@ -2897,7 +3905,13 @@
         <v>211</v>
       </c>
     </row>
-    <row r="148" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="148" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D148" s="1">
+        <v>8014</v>
+      </c>
+      <c r="E148" s="1" t="s">
+        <v>389</v>
+      </c>
       <c r="G148" s="1">
         <v>146</v>
       </c>
@@ -2905,7 +3919,13 @@
         <v>212</v>
       </c>
     </row>
-    <row r="149" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="149" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D149" s="1">
+        <v>8015</v>
+      </c>
+      <c r="E149" s="1" t="s">
+        <v>390</v>
+      </c>
       <c r="G149" s="1">
         <v>147</v>
       </c>
@@ -2913,7 +3933,13 @@
         <v>213</v>
       </c>
     </row>
-    <row r="150" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="150" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D150" s="1">
+        <v>8016</v>
+      </c>
+      <c r="E150" s="1" t="s">
+        <v>391</v>
+      </c>
       <c r="G150" s="1">
         <v>148</v>
       </c>
@@ -2921,7 +3947,13 @@
         <v>214</v>
       </c>
     </row>
-    <row r="151" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="151" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D151" s="1">
+        <v>9001</v>
+      </c>
+      <c r="E151" s="1" t="s">
+        <v>392</v>
+      </c>
       <c r="G151" s="1">
         <v>149</v>
       </c>
@@ -2929,7 +3961,13 @@
         <v>215</v>
       </c>
     </row>
-    <row r="152" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="152" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D152" s="1">
+        <v>9002</v>
+      </c>
+      <c r="E152" s="1" t="s">
+        <v>393</v>
+      </c>
       <c r="G152" s="1">
         <v>150</v>
       </c>
@@ -2937,7 +3975,13 @@
         <v>216</v>
       </c>
     </row>
-    <row r="153" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="153" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D153" s="1">
+        <v>9003</v>
+      </c>
+      <c r="E153" s="1" t="s">
+        <v>394</v>
+      </c>
       <c r="G153" s="1">
         <v>151</v>
       </c>
@@ -2945,7 +3989,13 @@
         <v>217</v>
       </c>
     </row>
-    <row r="154" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="154" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D154" s="1">
+        <v>9004</v>
+      </c>
+      <c r="E154" s="1" t="s">
+        <v>395</v>
+      </c>
       <c r="G154" s="1">
         <v>152</v>
       </c>
@@ -2953,7 +4003,13 @@
         <v>218</v>
       </c>
     </row>
-    <row r="155" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="155" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D155" s="1">
+        <v>9005</v>
+      </c>
+      <c r="E155" s="1" t="s">
+        <v>396</v>
+      </c>
       <c r="G155" s="1">
         <v>153</v>
       </c>
@@ -2961,7 +4017,13 @@
         <v>219</v>
       </c>
     </row>
-    <row r="156" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="156" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D156" s="1">
+        <v>9006</v>
+      </c>
+      <c r="E156" s="1" t="s">
+        <v>397</v>
+      </c>
       <c r="G156" s="1">
         <v>154</v>
       </c>
@@ -2969,7 +4031,13 @@
         <v>220</v>
       </c>
     </row>
-    <row r="157" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="157" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D157" s="1">
+        <v>9007</v>
+      </c>
+      <c r="E157" s="1" t="s">
+        <v>398</v>
+      </c>
       <c r="G157" s="1">
         <v>155</v>
       </c>
@@ -2977,7 +4045,13 @@
         <v>221</v>
       </c>
     </row>
-    <row r="158" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="158" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D158" s="1">
+        <v>9008</v>
+      </c>
+      <c r="E158" s="1" t="s">
+        <v>399</v>
+      </c>
       <c r="G158" s="1">
         <v>156</v>
       </c>
@@ -2985,7 +4059,13 @@
         <v>222</v>
       </c>
     </row>
-    <row r="159" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="159" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D159" s="1">
+        <v>9009</v>
+      </c>
+      <c r="E159" s="1" t="s">
+        <v>400</v>
+      </c>
       <c r="G159" s="1">
         <v>157</v>
       </c>
@@ -2993,7 +4073,13 @@
         <v>223</v>
       </c>
     </row>
-    <row r="160" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="160" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D160" s="1">
+        <v>9010</v>
+      </c>
+      <c r="E160" s="1" t="s">
+        <v>401</v>
+      </c>
       <c r="G160" s="1">
         <v>158</v>
       </c>
@@ -3001,7 +4087,13 @@
         <v>224</v>
       </c>
     </row>
-    <row r="161" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="161" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D161" s="1">
+        <v>9011</v>
+      </c>
+      <c r="E161" s="1" t="s">
+        <v>402</v>
+      </c>
       <c r="G161" s="1">
         <v>159</v>
       </c>
@@ -3009,7 +4101,13 @@
         <v>225</v>
       </c>
     </row>
-    <row r="162" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="162" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D162" s="1">
+        <v>9012</v>
+      </c>
+      <c r="E162" s="1" t="s">
+        <v>403</v>
+      </c>
       <c r="G162" s="1">
         <v>160</v>
       </c>
@@ -3017,7 +4115,13 @@
         <v>226</v>
       </c>
     </row>
-    <row r="163" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="163" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D163" s="1">
+        <v>9013</v>
+      </c>
+      <c r="E163" s="1" t="s">
+        <v>404</v>
+      </c>
       <c r="G163" s="1">
         <v>161</v>
       </c>
@@ -3025,7 +4129,13 @@
         <v>227</v>
       </c>
     </row>
-    <row r="164" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="164" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D164" s="1">
+        <v>9014</v>
+      </c>
+      <c r="E164" s="1" t="s">
+        <v>405</v>
+      </c>
       <c r="G164" s="1">
         <v>162</v>
       </c>
@@ -3033,7 +4143,13 @@
         <v>228</v>
       </c>
     </row>
-    <row r="165" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="165" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D165" s="1">
+        <v>9015</v>
+      </c>
+      <c r="E165" s="1" t="s">
+        <v>406</v>
+      </c>
       <c r="G165" s="1">
         <v>163</v>
       </c>
@@ -3041,7 +4157,13 @@
         <v>229</v>
       </c>
     </row>
-    <row r="166" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="166" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D166" s="1">
+        <v>9016</v>
+      </c>
+      <c r="E166" s="1" t="s">
+        <v>407</v>
+      </c>
       <c r="G166" s="1">
         <v>164</v>
       </c>
@@ -3049,7 +4171,13 @@
         <v>230</v>
       </c>
     </row>
-    <row r="167" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="167" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D167" s="1">
+        <v>9017</v>
+      </c>
+      <c r="E167" s="1" t="s">
+        <v>408</v>
+      </c>
       <c r="G167" s="1">
         <v>165</v>
       </c>
@@ -3057,7 +4185,13 @@
         <v>231</v>
       </c>
     </row>
-    <row r="168" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="168" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D168" s="1">
+        <v>9018</v>
+      </c>
+      <c r="E168" s="1" t="s">
+        <v>409</v>
+      </c>
       <c r="G168" s="1">
         <v>166</v>
       </c>
@@ -3065,7 +4199,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="169" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="169" spans="4:8" x14ac:dyDescent="0.3">
       <c r="G169" s="1">
         <v>167</v>
       </c>
@@ -3073,7 +4207,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="170" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="170" spans="4:8" x14ac:dyDescent="0.3">
       <c r="G170" s="1">
         <v>168</v>
       </c>
@@ -3081,7 +4215,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="171" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="171" spans="4:8" x14ac:dyDescent="0.3">
       <c r="G171" s="1">
         <v>169</v>
       </c>
@@ -3089,7 +4223,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="172" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="172" spans="4:8" x14ac:dyDescent="0.3">
       <c r="G172" s="1">
         <v>170</v>
       </c>
@@ -3097,7 +4231,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="173" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="173" spans="4:8" x14ac:dyDescent="0.3">
       <c r="G173" s="1">
         <v>171</v>
       </c>
@@ -3105,7 +4239,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="174" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="174" spans="4:8" x14ac:dyDescent="0.3">
       <c r="G174" s="1">
         <v>172</v>
       </c>
@@ -3113,7 +4247,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="175" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="175" spans="4:8" x14ac:dyDescent="0.3">
       <c r="G175" s="1">
         <v>173</v>
       </c>
@@ -3121,7 +4255,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="176" spans="7:8" x14ac:dyDescent="0.3">
+    <row r="176" spans="4:8" x14ac:dyDescent="0.3">
       <c r="G176" s="1">
         <v>174</v>
       </c>

</xml_diff>

<commit_message>
se arreglo el que no saliera el nombre del equipo
</commit_message>
<xml_diff>
--- a/Ids Ligas, Equipo.xlsx
+++ b/Ids Ligas, Equipo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MATEO\Videos\JAVASCRIPT\APIs\sports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3A65FE3-CAEA-405A-95B6-04E4C2C70239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1F3C5DF-1D66-4DBD-87A6-311D83715D78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{13C4450F-79C6-46C9-9EE9-A368FE75A248}"/>
+    <workbookView xWindow="10908" yWindow="3864" windowWidth="11172" windowHeight="7608" xr2:uid="{13C4450F-79C6-46C9-9EE9-A368FE75A248}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="413">
   <si>
     <t>id</t>
   </si>
@@ -1255,6 +1255,15 @@
   </si>
   <si>
     <t>Al Najma</t>
+  </si>
+  <si>
+    <t>Tercera Federación</t>
+  </si>
+  <si>
+    <t>Youth League</t>
+  </si>
+  <si>
+    <t>Primera Federación</t>
   </si>
 </sst>
 </file>
@@ -2268,6 +2277,12 @@
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>29</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>410</v>
+      </c>
       <c r="D31" s="1">
         <v>2008</v>
       </c>
@@ -2282,6 +2297,12 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" s="1">
+        <v>30</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>411</v>
+      </c>
       <c r="D32" s="1">
         <v>2009</v>
       </c>
@@ -2295,7 +2316,13 @@
         <v>96</v>
       </c>
     </row>
-    <row r="33" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="1">
+        <v>31</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>412</v>
+      </c>
       <c r="D33" s="1">
         <v>2010</v>
       </c>
@@ -2309,7 +2336,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="34" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D34" s="1">
         <v>2011</v>
       </c>
@@ -2323,7 +2350,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D35" s="1">
         <v>2012</v>
       </c>
@@ -2337,7 +2364,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="36" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D36" s="1">
         <v>2013</v>
       </c>
@@ -2351,7 +2378,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="37" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D37" s="1">
         <v>2014</v>
       </c>
@@ -2365,7 +2392,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="38" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D38" s="1">
         <v>2015</v>
       </c>
@@ -2379,7 +2406,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="39" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D39" s="1">
         <v>2016</v>
       </c>
@@ -2393,7 +2420,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="40" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D40" s="1">
         <v>2017</v>
       </c>
@@ -2407,7 +2434,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="41" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D41" s="1">
         <v>2018</v>
       </c>
@@ -2421,7 +2448,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="42" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D42" s="1">
         <v>2019</v>
       </c>
@@ -2435,7 +2462,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="43" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D43" s="1">
         <v>2020</v>
       </c>
@@ -2449,7 +2476,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="44" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D44" s="1">
         <v>3001</v>
       </c>
@@ -2463,7 +2490,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="45" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D45" s="1">
         <v>3002</v>
       </c>
@@ -2477,7 +2504,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="46" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D46" s="1">
         <v>3003</v>
       </c>
@@ -2491,7 +2518,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="47" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D47" s="1">
         <v>3004</v>
       </c>
@@ -2505,7 +2532,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="48" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D48" s="1">
         <v>3005</v>
       </c>

</xml_diff>

<commit_message>
se añadio nuevos datos
</commit_message>
<xml_diff>
--- a/Ids Ligas, Equipo.xlsx
+++ b/Ids Ligas, Equipo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29509"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29517"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MATEO\Videos\JAVASCRIPT\APIs\sports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{196A5E59-07CE-4758-B3A4-63F27450C87B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75290992-14B4-477A-A1AC-07382210F422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="684" yWindow="3624" windowWidth="11172" windowHeight="7608" xr2:uid="{13C4450F-79C6-46C9-9EE9-A368FE75A248}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="415">
   <si>
     <t>id</t>
   </si>
@@ -1267,9 +1267,6 @@
   </si>
   <si>
     <t>Concafac Champions Cup</t>
-  </si>
-  <si>
-    <t>ma</t>
   </si>
   <si>
     <t>Segunda Federación</t>
@@ -2138,8 +2135,8 @@
       <c r="E23" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>414</v>
+      <c r="G23" s="1">
+        <v>21</v>
       </c>
       <c r="H23" s="1" t="s">
         <v>87</v>
@@ -2370,7 +2367,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D35" s="1">
         <v>2012</v>

</xml_diff>